<commit_message>
fix(p1): align buyer files, print layouts and release checks
</commit_message>
<xml_diff>
--- a/products-storage/01-zakrytie-rabot/06-zhurnal-obemov.xlsx
+++ b/products-storage/01-zakrytie-rabot/06-zhurnal-obemov.xlsx
@@ -1,191 +1,281 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Реестр'!$A$3:$J$103</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="1" r:id="Rb0b392e47418407d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="2" r:id="R15398917a5e24894"/>
+  </x:sheets>
+</x:workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00242629"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00E85D22"/>
-      <sz val="16"/>
-    </font>
-  </fonts>
-  <fills count="4">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00242629"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E85D22"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="3">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="00B8B8B8"/>
-      </bottom>
-    </border>
-    <border>
-      <bottom style="hair">
-        <color rgb="00DDDDDD"/>
-      </bottom>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:fonts count="13">
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF242629"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFE85D22"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF2B2E31"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF2B2E31"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF62666A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF62666A"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF2B2E31"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF34383B"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="6">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF242629"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE85D22"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF34383B"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="4">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8B8B8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="hair">
+        <x:color rgb="FFDDDDDD"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFB49A65"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="22">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0"/>
+  </x:cellStyles>
+  <x:colors>
+    <x:indexedColors>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008000"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00808000"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="00C0C0C0"/>
+      <x:rgbColor rgb="00808080"/>
+      <x:rgbColor rgb="009999FF"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00FFFFCC"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00660066"/>
+      <x:rgbColor rgb="00FF8080"/>
+      <x:rgbColor rgb="000066CC"/>
+      <x:rgbColor rgb="00CCCCFF"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="0000CCFF"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00CCFFCC"/>
+      <x:rgbColor rgb="00FFFF99"/>
+      <x:rgbColor rgb="0099CCFF"/>
+      <x:rgbColor rgb="00FF99CC"/>
+      <x:rgbColor rgb="00CC99FF"/>
+      <x:rgbColor rgb="00FFCC99"/>
+      <x:rgbColor rgb="003366FF"/>
+      <x:rgbColor rgb="0033CCCC"/>
+      <x:rgbColor rgb="0099CC00"/>
+      <x:rgbColor rgb="00FFCC00"/>
+      <x:rgbColor rgb="00FF9900"/>
+      <x:rgbColor rgb="00FF6600"/>
+      <x:rgbColor rgb="00666699"/>
+      <x:rgbColor rgb="00969696"/>
+      <x:rgbColor rgb="00003366"/>
+      <x:rgbColor rgb="00339966"/>
+      <x:rgbColor rgb="00003300"/>
+      <x:rgbColor rgb="00333300"/>
+      <x:rgbColor rgb="00993300"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00333399"/>
+      <x:rgbColor rgb="00333333"/>
+    </x:indexedColors>
+  </x:colors>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -352,7 +442,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -361,13 +451,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -401,17 +491,6 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -466,95 +545,108 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <tabColor rgb="FFB49A65"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Журнал выполненных объёмов</t>
+          <t xml:space="preserve">Журнал выполненных объёмов</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+    </row>
+    <row r="2" ht="27" customHeight="1">
+      <c r="A2" s="16" t="str">
+        <v>Одна операция — одна строка. Заполните данные, затем отметьте результат и сохраните доказательства.</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Заполняйте одну операцию в одной строке. Серые колонки — исходные данные; оранжевые — контроль.</t>
+          <t xml:space="preserve">Дата</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>Дата</t>
+          <t xml:space="preserve">Вид работ</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Вид работ</t>
+          <t xml:space="preserve">Оси/участок</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>Оси/участок</t>
+          <t xml:space="preserve">Ед.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
-          <t>Ед.</t>
+          <t xml:space="preserve">Объём за день</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
-          <t>Объём за день</t>
+          <t xml:space="preserve">Накопительный объём</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Накопительный объём</t>
+          <t xml:space="preserve">Проект/смета</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
-          <t>Проект/смета</t>
+          <t xml:space="preserve">Фото/доказательство</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Фото/доказательство</t>
+          <t xml:space="preserve">Ответственный</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
         <is>
-          <t>Ответственный</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Примечание</t>
+          <t xml:space="preserve">Примечание</t>
         </is>
       </c>
     </row>
@@ -1759,42 +1851,41 @@
       <c r="J103" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J103"/>
-  <mergeCells count="2">
+  <mergeCells>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col min="1" max="1" width="75" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>Журнал выполненных объёмов</t>
+          <t xml:space="preserve">Журнал выполненных объёмов</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="3" ht="108" customHeight="1">
+      <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>1. Сделайте копию файла для объекта. 2. Назначьте владельца реестра. 3. Обновляйте статусы не реже двух раз в неделю. 4. Не удаляйте историю — меняйте статус и добавляйте комментарий. 5. Храните ссылки на доказательства передачи.</t>
+          <t xml:space="preserve">1. Сделайте копию файла для объекта. 2. Назначьте владельца реестра. 3. Обновляйте статусы не реже двух раз в неделю. 4. Не удаляйте историю — меняйте статус и добавляйте комментарий. 5. Храните ссылки на доказательства передачи.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>